<commit_message>
Add weekly All Salons file(s) (05/31/2026)
</commit_message>
<xml_diff>
--- a/All Salons 05.22.26.xlsx
+++ b/All Salons 05.22.26.xlsx
@@ -15,7 +15,7 @@
   <sheets>
     <sheet name="Export" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
@@ -524,9 +524,6 @@
   </cellStyles>
   <dxfs count="21">
     <dxf>
-      <alignment vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="165" formatCode="#,##0.0%;\-#,##0.0%;#,##0.0%"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -607,6 +604,9 @@
         </bottom>
       </border>
     </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -621,31 +621,31 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C7E371EF-E734-43CC-A665-30A22CAD5907}" name="Table1" displayName="Table1" ref="A1:S93" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C7E371EF-E734-43CC-A665-30A22CAD5907}" name="Table1" displayName="Table1" ref="A1:S93" totalsRowShown="0" headerRowDxfId="20" headerRowBorderDxfId="19">
   <autoFilter ref="A1:S93" xr:uid="{C7E371EF-E734-43CC-A665-30A22CAD5907}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:S93">
     <sortCondition ref="C1:C93"/>
   </sortState>
   <tableColumns count="19">
-    <tableColumn id="1" xr3:uid="{129C4BF4-9505-4F60-8FB4-E1DDDD073244}" name="Salon" dataDxfId="19"/>
-    <tableColumn id="2" xr3:uid="{866C3F98-3E3F-4F9E-8247-9AF44BC758F9}" name="SalonWeekEndingDate" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{98DC0DF4-1D5B-48DF-BCF6-DC354B5FE5E1}" name="Cust Count" dataDxfId="17"/>
-    <tableColumn id="4" xr3:uid="{4407F71B-D41B-4C49-BB07-533141EB9C9D}" name="Cust Count Last Year" dataDxfId="16"/>
-    <tableColumn id="5" xr3:uid="{09B6CB02-2185-44F3-8116-01D928E88F44}" name="Cust Count % Change" dataDxfId="15"/>
-    <tableColumn id="6" xr3:uid="{E2F8E600-1895-42A1-91AF-19A71293E079}" name="New Cust" dataDxfId="14"/>
-    <tableColumn id="7" xr3:uid="{3704A0BC-08C9-4E72-B6FC-B524C99F4E3A}" name="New Cust %" dataDxfId="13"/>
-    <tableColumn id="8" xr3:uid="{FD9EB296-CC50-4930-88B6-8E1C07AD120F}" name="Salon New Cust Return %" dataDxfId="12"/>
-    <tableColumn id="9" xr3:uid="{9EB7C997-38FE-4E7F-9C6F-9977B2FB9090}" name="Salon Repeat Cust Return %" dataDxfId="11"/>
-    <tableColumn id="10" xr3:uid="{1E6DB7EF-6442-4720-ACAD-4A81BB8ADBFF}" name="Floor Hours" dataDxfId="10"/>
-    <tableColumn id="11" xr3:uid="{9EDD6F29-2998-4C48-9C08-BD3B6AAC04AC}" name="Sat/Sun Floor Hours %" dataDxfId="9"/>
-    <tableColumn id="12" xr3:uid="{5DE97F0A-E975-4ED4-A803-060578BF0022}" name="Floor Hours Growth" dataDxfId="8"/>
-    <tableColumn id="13" xr3:uid="{3D07DD16-2ADD-4A07-9735-0621E3C62F04}" name="Wait Times &gt; 15Min %" dataDxfId="7"/>
-    <tableColumn id="14" xr3:uid="{04124BA1-04FF-468A-A511-EFB451DAF01F}" name="Sat/Sun Wait Times &gt; 15Min %" dataDxfId="6"/>
-    <tableColumn id="15" xr3:uid="{3EB838D9-B105-40AC-A80B-989D1CA87B4D}" name="Avg Wait Time" dataDxfId="5"/>
-    <tableColumn id="16" xr3:uid="{80FBD0E5-BB52-45C3-A793-685FBC04A735}" name="Avg HC Time" dataDxfId="4"/>
-    <tableColumn id="17" xr3:uid="{6F5C3AE1-D0C7-4EBD-BA0D-CF5062FC41E9}" name="CPH" dataDxfId="3"/>
-    <tableColumn id="18" xr3:uid="{C3D8869C-E68B-440F-A732-ECD8ADF070A2}" name="Productivity" dataDxfId="2"/>
-    <tableColumn id="19" xr3:uid="{99A04637-6617-4F5A-9EC9-0683428D3243}" name="Discount %" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{129C4BF4-9505-4F60-8FB4-E1DDDD073244}" name="Salon" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{866C3F98-3E3F-4F9E-8247-9AF44BC758F9}" name="SalonWeekEndingDate" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{98DC0DF4-1D5B-48DF-BCF6-DC354B5FE5E1}" name="Cust Count" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{4407F71B-D41B-4C49-BB07-533141EB9C9D}" name="Cust Count Last Year" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{09B6CB02-2185-44F3-8116-01D928E88F44}" name="Cust Count % Change" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{E2F8E600-1895-42A1-91AF-19A71293E079}" name="New Cust" dataDxfId="13"/>
+    <tableColumn id="7" xr3:uid="{3704A0BC-08C9-4E72-B6FC-B524C99F4E3A}" name="New Cust %" dataDxfId="12"/>
+    <tableColumn id="8" xr3:uid="{FD9EB296-CC50-4930-88B6-8E1C07AD120F}" name="Salon New Cust Return %" dataDxfId="11"/>
+    <tableColumn id="9" xr3:uid="{9EB7C997-38FE-4E7F-9C6F-9977B2FB9090}" name="Salon Repeat Cust Return %" dataDxfId="10"/>
+    <tableColumn id="10" xr3:uid="{1E6DB7EF-6442-4720-ACAD-4A81BB8ADBFF}" name="Floor Hours" dataDxfId="9"/>
+    <tableColumn id="11" xr3:uid="{9EDD6F29-2998-4C48-9C08-BD3B6AAC04AC}" name="Sat/Sun Floor Hours %" dataDxfId="8"/>
+    <tableColumn id="12" xr3:uid="{5DE97F0A-E975-4ED4-A803-060578BF0022}" name="Floor Hours Growth" dataDxfId="7"/>
+    <tableColumn id="13" xr3:uid="{3D07DD16-2ADD-4A07-9735-0621E3C62F04}" name="Wait Times &gt; 15Min %" dataDxfId="6"/>
+    <tableColumn id="14" xr3:uid="{04124BA1-04FF-468A-A511-EFB451DAF01F}" name="Sat/Sun Wait Times &gt; 15Min %" dataDxfId="5"/>
+    <tableColumn id="15" xr3:uid="{3EB838D9-B105-40AC-A80B-989D1CA87B4D}" name="Avg Wait Time" dataDxfId="4"/>
+    <tableColumn id="16" xr3:uid="{80FBD0E5-BB52-45C3-A793-685FBC04A735}" name="Avg HC Time" dataDxfId="3"/>
+    <tableColumn id="17" xr3:uid="{6F5C3AE1-D0C7-4EBD-BA0D-CF5062FC41E9}" name="CPH" dataDxfId="2"/>
+    <tableColumn id="18" xr3:uid="{C3D8869C-E68B-440F-A732-ECD8ADF070A2}" name="Productivity" dataDxfId="1"/>
+    <tableColumn id="19" xr3:uid="{99A04637-6617-4F5A-9EC9-0683428D3243}" name="Discount %" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>